<commit_message>
Fix SKU numbering: continue from SKU0277, not SKU0089
read_file_content returned a truncated view of the SKUs tab that stopped
at SKU0089, so the appended ids started at SKU0090 and would have
collided with 243 live rows. Exporting the workbook as xlsx instead shows
the tab really holds 332 rows: Giti patterns up to SKU0277, plus
LL0001-LL0049 for Linglong and a few category-prefixed ids.

New rows now run SKU0278-SKU0349, and the generator derives both the
header and the next id from the live sheet rather than from constants, so
a re-run after further edits stays correct. Adds assertions for id
collisions, id uniqueness and column count.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015Hfm3HvyUfCpK4wwTTpWTX
</commit_message>
<xml_diff>
--- a/data/rokudo_rows.xlsx
+++ b/data/rokudo_rows.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="rokudo rows" sheetId="1" r:id="rId1"/>
+    <sheet name="SKUs append" sheetId="1" r:id="rId1"/>
   </sheets>
 </workbook>
 </file>
@@ -512,7 +512,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>SKU0090</v>
+        <v>SKU0278</v>
       </c>
       <c r="B2" t="str">
         <v>tire</v>
@@ -545,7 +545,7 @@
         <v>8</v>
       </c>
       <c r="L2" t="str">
-        <v>Sentury pricelist 2026</v>
+        <v>SENTURY; New SKU 2026-09-04 - เพิ่มจากไฟล์ราคา ATV Sentury (ST_July)</v>
       </c>
       <c r="M2" t="str">
         <v/>
@@ -592,7 +592,7 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>SKU0091</v>
+        <v>SKU0279</v>
       </c>
       <c r="B3" t="str">
         <v>tire</v>
@@ -625,7 +625,7 @@
         <v>8</v>
       </c>
       <c r="L3" t="str">
-        <v>Sentury pricelist 2026</v>
+        <v>SENTURY; New SKU 2026-09-04 - เพิ่มจากไฟล์ราคา ATV Sentury (ST_July)</v>
       </c>
       <c r="M3" t="str">
         <v/>
@@ -672,7 +672,7 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>SKU0092</v>
+        <v>SKU0280</v>
       </c>
       <c r="B4" t="str">
         <v>tire</v>
@@ -705,7 +705,7 @@
         <v>8</v>
       </c>
       <c r="L4" t="str">
-        <v>Sentury pricelist 2026</v>
+        <v>SENTURY; New SKU 2026-09-04 - เพิ่มจากไฟล์ราคา ATV Sentury (ST_July)</v>
       </c>
       <c r="M4" t="str">
         <v/>
@@ -752,7 +752,7 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>SKU0093</v>
+        <v>SKU0281</v>
       </c>
       <c r="B5" t="str">
         <v>tire</v>
@@ -785,7 +785,7 @@
         <v>8</v>
       </c>
       <c r="L5" t="str">
-        <v>Sentury pricelist 2026</v>
+        <v>SENTURY; New SKU 2026-09-04 - เพิ่มจากไฟล์ราคา ATV Sentury (ST_July)</v>
       </c>
       <c r="M5" t="str">
         <v/>
@@ -832,7 +832,7 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>SKU0094</v>
+        <v>SKU0282</v>
       </c>
       <c r="B6" t="str">
         <v>tire</v>
@@ -865,7 +865,7 @@
         <v>8</v>
       </c>
       <c r="L6" t="str">
-        <v>Sentury pricelist 2026</v>
+        <v>SENTURY; New SKU 2026-09-04 - เพิ่มจากไฟล์ราคา ATV Sentury (ST_July)</v>
       </c>
       <c r="M6" t="str">
         <v/>
@@ -912,7 +912,7 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>SKU0095</v>
+        <v>SKU0283</v>
       </c>
       <c r="B7" t="str">
         <v>tire</v>
@@ -945,7 +945,7 @@
         <v>8</v>
       </c>
       <c r="L7" t="str">
-        <v>Sentury pricelist 2026</v>
+        <v>SENTURY; New SKU 2026-09-04 - เพิ่มจากไฟล์ราคา ATV Sentury (ST_July)</v>
       </c>
       <c r="M7" t="str">
         <v/>
@@ -992,7 +992,7 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>SKU0096</v>
+        <v>SKU0284</v>
       </c>
       <c r="B8" t="str">
         <v>tire</v>
@@ -1025,7 +1025,7 @@
         <v>8</v>
       </c>
       <c r="L8" t="str">
-        <v>Sentury pricelist 2026</v>
+        <v>SENTURY; New SKU 2026-09-04 - เพิ่มจากไฟล์ราคา ATV Sentury (ST_July)</v>
       </c>
       <c r="M8" t="str">
         <v/>
@@ -1072,7 +1072,7 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>SKU0097</v>
+        <v>SKU0285</v>
       </c>
       <c r="B9" t="str">
         <v>tire</v>
@@ -1105,7 +1105,7 @@
         <v>8</v>
       </c>
       <c r="L9" t="str">
-        <v>Sentury pricelist 2026</v>
+        <v>SENTURY; New SKU 2026-09-04 - เพิ่มจากไฟล์ราคา ATV Sentury (ST_July)</v>
       </c>
       <c r="M9" t="str">
         <v/>
@@ -1152,7 +1152,7 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>SKU0098</v>
+        <v>SKU0286</v>
       </c>
       <c r="B10" t="str">
         <v>tire</v>
@@ -1185,7 +1185,7 @@
         <v>8</v>
       </c>
       <c r="L10" t="str">
-        <v>Sentury pricelist 2026</v>
+        <v>SENTURY; New SKU 2026-09-04 - เพิ่มจากไฟล์ราคา ATV Sentury (ST_July)</v>
       </c>
       <c r="M10" t="str">
         <v/>
@@ -1232,7 +1232,7 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>SKU0099</v>
+        <v>SKU0287</v>
       </c>
       <c r="B11" t="str">
         <v>tire</v>
@@ -1265,7 +1265,7 @@
         <v>8</v>
       </c>
       <c r="L11" t="str">
-        <v>Sentury pricelist 2026</v>
+        <v>SENTURY; New SKU 2026-09-04 - เพิ่มจากไฟล์ราคา ATV Sentury (ST_July)</v>
       </c>
       <c r="M11" t="str">
         <v/>
@@ -1312,7 +1312,7 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>SKU0100</v>
+        <v>SKU0288</v>
       </c>
       <c r="B12" t="str">
         <v>tire</v>
@@ -1345,7 +1345,7 @@
         <v>8</v>
       </c>
       <c r="L12" t="str">
-        <v>Sentury pricelist 2026</v>
+        <v>SENTURY; New SKU 2026-09-04 - เพิ่มจากไฟล์ราคา ATV Sentury (ST_July)</v>
       </c>
       <c r="M12" t="str">
         <v/>
@@ -1392,7 +1392,7 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>SKU0101</v>
+        <v>SKU0289</v>
       </c>
       <c r="B13" t="str">
         <v>tire</v>
@@ -1425,7 +1425,7 @@
         <v>8</v>
       </c>
       <c r="L13" t="str">
-        <v>Sentury pricelist 2026</v>
+        <v>SENTURY; New SKU 2026-09-04 - เพิ่มจากไฟล์ราคา ATV Sentury (ST_July)</v>
       </c>
       <c r="M13" t="str">
         <v/>
@@ -1472,7 +1472,7 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>SKU0102</v>
+        <v>SKU0290</v>
       </c>
       <c r="B14" t="str">
         <v>tire</v>
@@ -1505,7 +1505,7 @@
         <v>8</v>
       </c>
       <c r="L14" t="str">
-        <v>Sentury pricelist 2026</v>
+        <v>SENTURY; New SKU 2026-09-04 - เพิ่มจากไฟล์ราคา ATV Sentury (ST_July)</v>
       </c>
       <c r="M14" t="str">
         <v/>
@@ -1552,7 +1552,7 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>SKU0103</v>
+        <v>SKU0291</v>
       </c>
       <c r="B15" t="str">
         <v>tire</v>
@@ -1585,7 +1585,7 @@
         <v>8</v>
       </c>
       <c r="L15" t="str">
-        <v>Sentury pricelist 2026</v>
+        <v>SENTURY; New SKU 2026-09-04 - เพิ่มจากไฟล์ราคา ATV Sentury (ST_July)</v>
       </c>
       <c r="M15" t="str">
         <v/>
@@ -1632,7 +1632,7 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>SKU0104</v>
+        <v>SKU0292</v>
       </c>
       <c r="B16" t="str">
         <v>tire</v>
@@ -1665,7 +1665,7 @@
         <v>8</v>
       </c>
       <c r="L16" t="str">
-        <v>Sentury pricelist 2026</v>
+        <v>SENTURY; New SKU 2026-09-04 - เพิ่มจากไฟล์ราคา ATV Sentury (ST_July)</v>
       </c>
       <c r="M16" t="str">
         <v/>
@@ -1712,7 +1712,7 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>SKU0105</v>
+        <v>SKU0293</v>
       </c>
       <c r="B17" t="str">
         <v>tire</v>
@@ -1745,7 +1745,7 @@
         <v>8</v>
       </c>
       <c r="L17" t="str">
-        <v>Sentury pricelist 2026</v>
+        <v>SENTURY; New SKU 2026-09-04 - เพิ่มจากไฟล์ราคา ATV Sentury (ST_July)</v>
       </c>
       <c r="M17" t="str">
         <v/>
@@ -1792,7 +1792,7 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>SKU0106</v>
+        <v>SKU0294</v>
       </c>
       <c r="B18" t="str">
         <v>tire</v>
@@ -1825,7 +1825,7 @@
         <v>8</v>
       </c>
       <c r="L18" t="str">
-        <v>Sentury pricelist 2026</v>
+        <v>SENTURY; New SKU 2026-09-04 - เพิ่มจากไฟล์ราคา ATV Sentury (ST_July)</v>
       </c>
       <c r="M18" t="str">
         <v/>
@@ -1872,7 +1872,7 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>SKU0107</v>
+        <v>SKU0295</v>
       </c>
       <c r="B19" t="str">
         <v>tire</v>
@@ -1905,7 +1905,7 @@
         <v>8</v>
       </c>
       <c r="L19" t="str">
-        <v>Sentury pricelist 2026</v>
+        <v>SENTURY; New SKU 2026-09-04 - เพิ่มจากไฟล์ราคา ATV Sentury (ST_July)</v>
       </c>
       <c r="M19" t="str">
         <v/>
@@ -1952,7 +1952,7 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>SKU0108</v>
+        <v>SKU0296</v>
       </c>
       <c r="B20" t="str">
         <v>tire</v>
@@ -1985,7 +1985,7 @@
         <v>8</v>
       </c>
       <c r="L20" t="str">
-        <v>Sentury pricelist 2026</v>
+        <v>SENTURY; New SKU 2026-09-04 - เพิ่มจากไฟล์ราคา ATV Sentury (ST_July)</v>
       </c>
       <c r="M20" t="str">
         <v/>
@@ -2032,7 +2032,7 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>SKU0109</v>
+        <v>SKU0297</v>
       </c>
       <c r="B21" t="str">
         <v>tire</v>
@@ -2065,7 +2065,7 @@
         <v>8</v>
       </c>
       <c r="L21" t="str">
-        <v>Sentury pricelist 2026</v>
+        <v>SENTURY; New SKU 2026-09-04 - เพิ่มจากไฟล์ราคา ATV Sentury (ST_July)</v>
       </c>
       <c r="M21" t="str">
         <v/>
@@ -2112,7 +2112,7 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>SKU0110</v>
+        <v>SKU0298</v>
       </c>
       <c r="B22" t="str">
         <v>tire</v>
@@ -2145,7 +2145,7 @@
         <v>8</v>
       </c>
       <c r="L22" t="str">
-        <v>Sentury pricelist 2026</v>
+        <v>SENTURY; New SKU 2026-09-04 - เพิ่มจากไฟล์ราคา ATV Sentury (ST_July)</v>
       </c>
       <c r="M22" t="str">
         <v/>
@@ -2192,7 +2192,7 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>SKU0111</v>
+        <v>SKU0299</v>
       </c>
       <c r="B23" t="str">
         <v>tire</v>
@@ -2225,7 +2225,7 @@
         <v>8</v>
       </c>
       <c r="L23" t="str">
-        <v>Sentury pricelist 2026</v>
+        <v>SENTURY; New SKU 2026-09-04 - เพิ่มจากไฟล์ราคา ATV Sentury (ST_July)</v>
       </c>
       <c r="M23" t="str">
         <v/>
@@ -2272,7 +2272,7 @@
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>SKU0112</v>
+        <v>SKU0300</v>
       </c>
       <c r="B24" t="str">
         <v>tire</v>
@@ -2305,7 +2305,7 @@
         <v>8</v>
       </c>
       <c r="L24" t="str">
-        <v>Sentury pricelist 2026</v>
+        <v>SENTURY; New SKU 2026-09-04 - เพิ่มจากไฟล์ราคา ATV Sentury (ST_July)</v>
       </c>
       <c r="M24" t="str">
         <v/>
@@ -2352,7 +2352,7 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>SKU0113</v>
+        <v>SKU0301</v>
       </c>
       <c r="B25" t="str">
         <v>tire</v>
@@ -2385,7 +2385,7 @@
         <v>8</v>
       </c>
       <c r="L25" t="str">
-        <v>Sentury pricelist 2026</v>
+        <v>SENTURY; New SKU 2026-09-04 - เพิ่มจากไฟล์ราคา ATV Sentury (ST_July)</v>
       </c>
       <c r="M25" t="str">
         <v/>
@@ -2432,7 +2432,7 @@
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>SKU0114</v>
+        <v>SKU0302</v>
       </c>
       <c r="B26" t="str">
         <v>tire</v>
@@ -2465,7 +2465,7 @@
         <v>8</v>
       </c>
       <c r="L26" t="str">
-        <v>Sentury pricelist 2026</v>
+        <v>SENTURY; New SKU 2026-09-04 - เพิ่มจากไฟล์ราคา ATV Sentury (ST_July)</v>
       </c>
       <c r="M26" t="str">
         <v/>
@@ -2512,7 +2512,7 @@
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>SKU0115</v>
+        <v>SKU0303</v>
       </c>
       <c r="B27" t="str">
         <v>tire</v>
@@ -2545,7 +2545,7 @@
         <v>8</v>
       </c>
       <c r="L27" t="str">
-        <v>Sentury pricelist 2026</v>
+        <v>SENTURY; New SKU 2026-09-04 - เพิ่มจากไฟล์ราคา ATV Sentury (ST_July)</v>
       </c>
       <c r="M27" t="str">
         <v/>
@@ -2592,7 +2592,7 @@
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>SKU0116</v>
+        <v>SKU0304</v>
       </c>
       <c r="B28" t="str">
         <v>tire</v>
@@ -2625,7 +2625,7 @@
         <v>8</v>
       </c>
       <c r="L28" t="str">
-        <v>Sentury pricelist 2026</v>
+        <v>SENTURY; New SKU 2026-09-04 - เพิ่มจากไฟล์ราคา ATV Sentury (ST_July)</v>
       </c>
       <c r="M28" t="str">
         <v/>
@@ -2672,7 +2672,7 @@
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>SKU0117</v>
+        <v>SKU0305</v>
       </c>
       <c r="B29" t="str">
         <v>tire</v>
@@ -2705,7 +2705,7 @@
         <v>8</v>
       </c>
       <c r="L29" t="str">
-        <v>Sentury pricelist 2026</v>
+        <v>SENTURY; New SKU 2026-09-04 - เพิ่มจากไฟล์ราคา ATV Sentury (ST_July)</v>
       </c>
       <c r="M29" t="str">
         <v/>
@@ -2752,7 +2752,7 @@
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>SKU0118</v>
+        <v>SKU0306</v>
       </c>
       <c r="B30" t="str">
         <v>tire</v>
@@ -2785,7 +2785,7 @@
         <v>8</v>
       </c>
       <c r="L30" t="str">
-        <v>Sentury pricelist 2026</v>
+        <v>SENTURY; New SKU 2026-09-04 - เพิ่มจากไฟล์ราคา ATV Sentury (ST_July)</v>
       </c>
       <c r="M30" t="str">
         <v/>
@@ -2832,7 +2832,7 @@
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>SKU0119</v>
+        <v>SKU0307</v>
       </c>
       <c r="B31" t="str">
         <v>tire</v>
@@ -2865,7 +2865,7 @@
         <v>8</v>
       </c>
       <c r="L31" t="str">
-        <v>Sentury pricelist 2026</v>
+        <v>SENTURY; New SKU 2026-09-04 - เพิ่มจากไฟล์ราคา ATV Sentury (ST_July)</v>
       </c>
       <c r="M31" t="str">
         <v/>
@@ -2912,7 +2912,7 @@
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>SKU0120</v>
+        <v>SKU0308</v>
       </c>
       <c r="B32" t="str">
         <v>tire</v>
@@ -2945,7 +2945,7 @@
         <v>8</v>
       </c>
       <c r="L32" t="str">
-        <v>WL; Sentury pricelist 2026</v>
+        <v>WL; SENTURY; New SKU 2026-09-04 - เพิ่มจากไฟล์ราคา ATV Sentury (ST_July)</v>
       </c>
       <c r="M32" t="str">
         <v/>
@@ -2992,7 +2992,7 @@
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>SKU0121</v>
+        <v>SKU0309</v>
       </c>
       <c r="B33" t="str">
         <v>tire</v>
@@ -3025,7 +3025,7 @@
         <v>8</v>
       </c>
       <c r="L33" t="str">
-        <v>WL; Sentury pricelist 2026</v>
+        <v>WL; SENTURY; New SKU 2026-09-04 - เพิ่มจากไฟล์ราคา ATV Sentury (ST_July)</v>
       </c>
       <c r="M33" t="str">
         <v/>
@@ -3072,7 +3072,7 @@
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>SKU0122</v>
+        <v>SKU0310</v>
       </c>
       <c r="B34" t="str">
         <v>tire</v>
@@ -3105,7 +3105,7 @@
         <v>8</v>
       </c>
       <c r="L34" t="str">
-        <v>WL; Sentury pricelist 2026</v>
+        <v>WL; SENTURY; New SKU 2026-09-04 - เพิ่มจากไฟล์ราคา ATV Sentury (ST_July)</v>
       </c>
       <c r="M34" t="str">
         <v/>
@@ -3152,7 +3152,7 @@
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>SKU0123</v>
+        <v>SKU0311</v>
       </c>
       <c r="B35" t="str">
         <v>tire</v>
@@ -3185,7 +3185,7 @@
         <v>8</v>
       </c>
       <c r="L35" t="str">
-        <v>WL; Sentury pricelist 2026</v>
+        <v>WL; SENTURY; New SKU 2026-09-04 - เพิ่มจากไฟล์ราคา ATV Sentury (ST_July)</v>
       </c>
       <c r="M35" t="str">
         <v/>
@@ -3232,7 +3232,7 @@
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>SKU0124</v>
+        <v>SKU0312</v>
       </c>
       <c r="B36" t="str">
         <v>tire</v>
@@ -3265,7 +3265,7 @@
         <v>8</v>
       </c>
       <c r="L36" t="str">
-        <v>WL; Sentury pricelist 2026</v>
+        <v>WL; SENTURY; New SKU 2026-09-04 - เพิ่มจากไฟล์ราคา ATV Sentury (ST_July)</v>
       </c>
       <c r="M36" t="str">
         <v/>
@@ -3312,7 +3312,7 @@
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>SKU0125</v>
+        <v>SKU0313</v>
       </c>
       <c r="B37" t="str">
         <v>tire</v>
@@ -3345,7 +3345,7 @@
         <v>8</v>
       </c>
       <c r="L37" t="str">
-        <v>WL; Sentury pricelist 2026</v>
+        <v>WL; SENTURY; New SKU 2026-09-04 - เพิ่มจากไฟล์ราคา ATV Sentury (ST_July)</v>
       </c>
       <c r="M37" t="str">
         <v/>
@@ -3392,7 +3392,7 @@
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>SKU0126</v>
+        <v>SKU0314</v>
       </c>
       <c r="B38" t="str">
         <v>tire</v>
@@ -3425,7 +3425,7 @@
         <v>8</v>
       </c>
       <c r="L38" t="str">
-        <v>WL; Sentury pricelist 2026</v>
+        <v>WL; SENTURY; New SKU 2026-09-04 - เพิ่มจากไฟล์ราคา ATV Sentury (ST_July)</v>
       </c>
       <c r="M38" t="str">
         <v/>
@@ -3472,7 +3472,7 @@
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>SKU0127</v>
+        <v>SKU0315</v>
       </c>
       <c r="B39" t="str">
         <v>tire</v>
@@ -3505,7 +3505,7 @@
         <v>8</v>
       </c>
       <c r="L39" t="str">
-        <v>WL; Sentury pricelist 2026</v>
+        <v>WL; SENTURY; New SKU 2026-09-04 - เพิ่มจากไฟล์ราคา ATV Sentury (ST_July)</v>
       </c>
       <c r="M39" t="str">
         <v/>
@@ -3552,7 +3552,7 @@
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>SKU0128</v>
+        <v>SKU0316</v>
       </c>
       <c r="B40" t="str">
         <v>tire</v>
@@ -3585,7 +3585,7 @@
         <v>8</v>
       </c>
       <c r="L40" t="str">
-        <v>WL; Sentury pricelist 2026</v>
+        <v>WL; SENTURY; New SKU 2026-09-04 - เพิ่มจากไฟล์ราคา ATV Sentury (ST_July)</v>
       </c>
       <c r="M40" t="str">
         <v/>
@@ -3632,7 +3632,7 @@
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>SKU0129</v>
+        <v>SKU0317</v>
       </c>
       <c r="B41" t="str">
         <v>tire</v>
@@ -3665,7 +3665,7 @@
         <v>8</v>
       </c>
       <c r="L41" t="str">
-        <v>WL; Sentury pricelist 2026</v>
+        <v>WL; SENTURY; New SKU 2026-09-04 - เพิ่มจากไฟล์ราคา ATV Sentury (ST_July)</v>
       </c>
       <c r="M41" t="str">
         <v/>
@@ -3712,7 +3712,7 @@
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>SKU0130</v>
+        <v>SKU0318</v>
       </c>
       <c r="B42" t="str">
         <v>tire</v>
@@ -3745,7 +3745,7 @@
         <v>8</v>
       </c>
       <c r="L42" t="str">
-        <v>WL; Sentury pricelist 2026</v>
+        <v>WL; SENTURY; New SKU 2026-09-04 - เพิ่มจากไฟล์ราคา ATV Sentury (ST_July)</v>
       </c>
       <c r="M42" t="str">
         <v/>
@@ -3792,7 +3792,7 @@
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>SKU0131</v>
+        <v>SKU0319</v>
       </c>
       <c r="B43" t="str">
         <v>tire</v>
@@ -3825,7 +3825,7 @@
         <v>8</v>
       </c>
       <c r="L43" t="str">
-        <v>WL; Sentury pricelist 2026</v>
+        <v>WL; SENTURY; New SKU 2026-09-04 - เพิ่มจากไฟล์ราคา ATV Sentury (ST_July)</v>
       </c>
       <c r="M43" t="str">
         <v/>
@@ -3872,7 +3872,7 @@
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>SKU0132</v>
+        <v>SKU0320</v>
       </c>
       <c r="B44" t="str">
         <v>tire</v>
@@ -3905,7 +3905,7 @@
         <v>8</v>
       </c>
       <c r="L44" t="str">
-        <v>WL; Sentury pricelist 2026</v>
+        <v>WL; SENTURY; New SKU 2026-09-04 - เพิ่มจากไฟล์ราคา ATV Sentury (ST_July)</v>
       </c>
       <c r="M44" t="str">
         <v/>
@@ -3952,7 +3952,7 @@
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>SKU0133</v>
+        <v>SKU0321</v>
       </c>
       <c r="B45" t="str">
         <v>tire</v>
@@ -3985,7 +3985,7 @@
         <v>8</v>
       </c>
       <c r="L45" t="str">
-        <v>Sentury pricelist 2026</v>
+        <v>SENTURY; New SKU 2026-09-04 - เพิ่มจากไฟล์ราคา ATV Sentury (ST_July)</v>
       </c>
       <c r="M45" t="str">
         <v/>
@@ -4032,7 +4032,7 @@
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>SKU0134</v>
+        <v>SKU0322</v>
       </c>
       <c r="B46" t="str">
         <v>tire</v>
@@ -4065,7 +4065,7 @@
         <v>8</v>
       </c>
       <c r="L46" t="str">
-        <v>Sentury pricelist 2026</v>
+        <v>SENTURY; New SKU 2026-09-04 - เพิ่มจากไฟล์ราคา ATV Sentury (ST_July)</v>
       </c>
       <c r="M46" t="str">
         <v/>
@@ -4112,7 +4112,7 @@
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>SKU0135</v>
+        <v>SKU0323</v>
       </c>
       <c r="B47" t="str">
         <v>tire</v>
@@ -4145,7 +4145,7 @@
         <v>8</v>
       </c>
       <c r="L47" t="str">
-        <v>Sentury pricelist 2026</v>
+        <v>SENTURY; New SKU 2026-09-04 - เพิ่มจากไฟล์ราคา ATV Sentury (ST_July)</v>
       </c>
       <c r="M47" t="str">
         <v/>
@@ -4192,7 +4192,7 @@
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>SKU0136</v>
+        <v>SKU0324</v>
       </c>
       <c r="B48" t="str">
         <v>tire</v>
@@ -4225,7 +4225,7 @@
         <v>8</v>
       </c>
       <c r="L48" t="str">
-        <v>Sentury pricelist 2026</v>
+        <v>SENTURY; New SKU 2026-09-04 - เพิ่มจากไฟล์ราคา ATV Sentury (ST_July)</v>
       </c>
       <c r="M48" t="str">
         <v/>
@@ -4272,7 +4272,7 @@
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>SKU0137</v>
+        <v>SKU0325</v>
       </c>
       <c r="B49" t="str">
         <v>tire</v>
@@ -4305,7 +4305,7 @@
         <v>8</v>
       </c>
       <c r="L49" t="str">
-        <v>Sentury pricelist 2026</v>
+        <v>SENTURY; New SKU 2026-09-04 - เพิ่มจากไฟล์ราคา ATV Sentury (ST_July)</v>
       </c>
       <c r="M49" t="str">
         <v/>
@@ -4352,7 +4352,7 @@
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>SKU0138</v>
+        <v>SKU0326</v>
       </c>
       <c r="B50" t="str">
         <v>tire</v>
@@ -4385,7 +4385,7 @@
         <v>8</v>
       </c>
       <c r="L50" t="str">
-        <v>Sentury pricelist 2026</v>
+        <v>SENTURY; New SKU 2026-09-04 - เพิ่มจากไฟล์ราคา ATV Sentury (ST_July)</v>
       </c>
       <c r="M50" t="str">
         <v/>
@@ -4432,7 +4432,7 @@
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>SKU0139</v>
+        <v>SKU0327</v>
       </c>
       <c r="B51" t="str">
         <v>tire</v>
@@ -4465,7 +4465,7 @@
         <v>8</v>
       </c>
       <c r="L51" t="str">
-        <v>Sentury pricelist 2026</v>
+        <v>SENTURY; New SKU 2026-09-04 - เพิ่มจากไฟล์ราคา ATV Sentury (ST_July)</v>
       </c>
       <c r="M51" t="str">
         <v/>
@@ -4512,7 +4512,7 @@
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>SKU0140</v>
+        <v>SKU0328</v>
       </c>
       <c r="B52" t="str">
         <v>tire</v>
@@ -4545,7 +4545,7 @@
         <v>8</v>
       </c>
       <c r="L52" t="str">
-        <v>Sentury pricelist 2026</v>
+        <v>SENTURY; New SKU 2026-09-04 - เพิ่มจากไฟล์ราคา ATV Sentury (ST_July)</v>
       </c>
       <c r="M52" t="str">
         <v/>
@@ -4592,7 +4592,7 @@
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>SKU0141</v>
+        <v>SKU0329</v>
       </c>
       <c r="B53" t="str">
         <v>tire</v>
@@ -4625,7 +4625,7 @@
         <v>8</v>
       </c>
       <c r="L53" t="str">
-        <v>Sentury pricelist 2026</v>
+        <v>SENTURY; New SKU 2026-09-04 - เพิ่มจากไฟล์ราคา ATV Sentury (ST_July)</v>
       </c>
       <c r="M53" t="str">
         <v/>
@@ -4672,7 +4672,7 @@
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>SKU0142</v>
+        <v>SKU0330</v>
       </c>
       <c r="B54" t="str">
         <v>tire</v>
@@ -4705,7 +4705,7 @@
         <v>8</v>
       </c>
       <c r="L54" t="str">
-        <v>Sentury pricelist 2026</v>
+        <v>SENTURY; New SKU 2026-09-04 - เพิ่มจากไฟล์ราคา ATV Sentury (ST_July)</v>
       </c>
       <c r="M54" t="str">
         <v/>
@@ -4752,7 +4752,7 @@
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>SKU0143</v>
+        <v>SKU0331</v>
       </c>
       <c r="B55" t="str">
         <v>tire</v>
@@ -4785,7 +4785,7 @@
         <v>8</v>
       </c>
       <c r="L55" t="str">
-        <v>Sentury pricelist 2026</v>
+        <v>SENTURY; New SKU 2026-09-04 - เพิ่มจากไฟล์ราคา ATV Sentury (ST_July)</v>
       </c>
       <c r="M55" t="str">
         <v/>
@@ -4832,7 +4832,7 @@
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>SKU0144</v>
+        <v>SKU0332</v>
       </c>
       <c r="B56" t="str">
         <v>tire</v>
@@ -4865,7 +4865,7 @@
         <v>8</v>
       </c>
       <c r="L56" t="str">
-        <v>Sentury pricelist 2026</v>
+        <v>SENTURY; New SKU 2026-09-04 - เพิ่มจากไฟล์ราคา ATV Sentury (ST_July)</v>
       </c>
       <c r="M56" t="str">
         <v/>
@@ -4912,7 +4912,7 @@
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>SKU0145</v>
+        <v>SKU0333</v>
       </c>
       <c r="B57" t="str">
         <v>tire</v>
@@ -4945,7 +4945,7 @@
         <v>8</v>
       </c>
       <c r="L57" t="str">
-        <v>Sentury pricelist 2026</v>
+        <v>SENTURY; New SKU 2026-09-04 - เพิ่มจากไฟล์ราคา ATV Sentury (ST_July)</v>
       </c>
       <c r="M57" t="str">
         <v/>
@@ -4992,7 +4992,7 @@
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>SKU0146</v>
+        <v>SKU0334</v>
       </c>
       <c r="B58" t="str">
         <v>tire</v>
@@ -5025,7 +5025,7 @@
         <v>8</v>
       </c>
       <c r="L58" t="str">
-        <v>Sentury pricelist 2026</v>
+        <v>SENTURY; New SKU 2026-09-04 - เพิ่มจากไฟล์ราคา ATV Sentury (ST_July)</v>
       </c>
       <c r="M58" t="str">
         <v/>
@@ -5072,7 +5072,7 @@
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>SKU0147</v>
+        <v>SKU0335</v>
       </c>
       <c r="B59" t="str">
         <v>tire</v>
@@ -5105,7 +5105,7 @@
         <v>8</v>
       </c>
       <c r="L59" t="str">
-        <v>Sentury pricelist 2026</v>
+        <v>SENTURY; New SKU 2026-09-04 - เพิ่มจากไฟล์ราคา ATV Sentury (ST_July)</v>
       </c>
       <c r="M59" t="str">
         <v/>
@@ -5152,7 +5152,7 @@
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>SKU0148</v>
+        <v>SKU0336</v>
       </c>
       <c r="B60" t="str">
         <v>tire</v>
@@ -5185,7 +5185,7 @@
         <v>8</v>
       </c>
       <c r="L60" t="str">
-        <v>Sentury pricelist 2026</v>
+        <v>SENTURY; New SKU 2026-09-04 - เพิ่มจากไฟล์ราคา ATV Sentury (ST_July)</v>
       </c>
       <c r="M60" t="str">
         <v/>
@@ -5232,7 +5232,7 @@
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>SKU0149</v>
+        <v>SKU0337</v>
       </c>
       <c r="B61" t="str">
         <v>tire</v>
@@ -5265,7 +5265,7 @@
         <v>8</v>
       </c>
       <c r="L61" t="str">
-        <v>Sentury pricelist 2026</v>
+        <v>SENTURY; New SKU 2026-09-04 - เพิ่มจากไฟล์ราคา ATV Sentury (ST_July)</v>
       </c>
       <c r="M61" t="str">
         <v/>
@@ -5312,7 +5312,7 @@
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v>SKU0150</v>
+        <v>SKU0338</v>
       </c>
       <c r="B62" t="str">
         <v>tire</v>
@@ -5345,7 +5345,7 @@
         <v>8</v>
       </c>
       <c r="L62" t="str">
-        <v>Sentury pricelist 2026</v>
+        <v>SENTURY; New SKU 2026-09-04 - เพิ่มจากไฟล์ราคา ATV Sentury (ST_July)</v>
       </c>
       <c r="M62" t="str">
         <v/>
@@ -5392,7 +5392,7 @@
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v>SKU0151</v>
+        <v>SKU0339</v>
       </c>
       <c r="B63" t="str">
         <v>tire</v>
@@ -5425,7 +5425,7 @@
         <v>8</v>
       </c>
       <c r="L63" t="str">
-        <v>Sentury pricelist 2026</v>
+        <v>SENTURY; New SKU 2026-09-04 - เพิ่มจากไฟล์ราคา ATV Sentury (ST_July)</v>
       </c>
       <c r="M63" t="str">
         <v/>
@@ -5472,7 +5472,7 @@
     </row>
     <row r="64">
       <c r="A64" t="str">
-        <v>SKU0152</v>
+        <v>SKU0340</v>
       </c>
       <c r="B64" t="str">
         <v>tire</v>
@@ -5505,7 +5505,7 @@
         <v>8</v>
       </c>
       <c r="L64" t="str">
-        <v>Sentury pricelist 2026</v>
+        <v>SENTURY; New SKU 2026-09-04 - เพิ่มจากไฟล์ราคา ATV Sentury (ST_July)</v>
       </c>
       <c r="M64" t="str">
         <v/>
@@ -5552,7 +5552,7 @@
     </row>
     <row r="65">
       <c r="A65" t="str">
-        <v>SKU0153</v>
+        <v>SKU0341</v>
       </c>
       <c r="B65" t="str">
         <v>tire</v>
@@ -5585,7 +5585,7 @@
         <v>8</v>
       </c>
       <c r="L65" t="str">
-        <v>Sentury pricelist 2026</v>
+        <v>SENTURY; New SKU 2026-09-04 - เพิ่มจากไฟล์ราคา ATV Sentury (ST_July)</v>
       </c>
       <c r="M65" t="str">
         <v/>
@@ -5632,7 +5632,7 @@
     </row>
     <row r="66">
       <c r="A66" t="str">
-        <v>SKU0154</v>
+        <v>SKU0342</v>
       </c>
       <c r="B66" t="str">
         <v>tire</v>
@@ -5665,7 +5665,7 @@
         <v>8</v>
       </c>
       <c r="L66" t="str">
-        <v>Sentury pricelist 2026</v>
+        <v>SENTURY; New SKU 2026-09-04 - เพิ่มจากไฟล์ราคา ATV Sentury (ST_July)</v>
       </c>
       <c r="M66" t="str">
         <v/>
@@ -5712,7 +5712,7 @@
     </row>
     <row r="67">
       <c r="A67" t="str">
-        <v>SKU0155</v>
+        <v>SKU0343</v>
       </c>
       <c r="B67" t="str">
         <v>tire</v>
@@ -5745,7 +5745,7 @@
         <v>8</v>
       </c>
       <c r="L67" t="str">
-        <v>Sentury pricelist 2026</v>
+        <v>SENTURY; New SKU 2026-09-04 - เพิ่มจากไฟล์ราคา ATV Sentury (ST_July)</v>
       </c>
       <c r="M67" t="str">
         <v/>
@@ -5792,7 +5792,7 @@
     </row>
     <row r="68">
       <c r="A68" t="str">
-        <v>SKU0156</v>
+        <v>SKU0344</v>
       </c>
       <c r="B68" t="str">
         <v>tire</v>
@@ -5825,7 +5825,7 @@
         <v>8</v>
       </c>
       <c r="L68" t="str">
-        <v>Sentury pricelist 2026</v>
+        <v>SENTURY; New SKU 2026-09-04 - เพิ่มจากไฟล์ราคา ATV Sentury (ST_July)</v>
       </c>
       <c r="M68" t="str">
         <v/>
@@ -5872,7 +5872,7 @@
     </row>
     <row r="69">
       <c r="A69" t="str">
-        <v>SKU0157</v>
+        <v>SKU0345</v>
       </c>
       <c r="B69" t="str">
         <v>tire</v>
@@ -5905,7 +5905,7 @@
         <v>8</v>
       </c>
       <c r="L69" t="str">
-        <v>Sentury pricelist 2026</v>
+        <v>SENTURY; New SKU 2026-09-04 - เพิ่มจากไฟล์ราคา ATV Sentury (ST_July)</v>
       </c>
       <c r="M69" t="str">
         <v/>
@@ -5952,7 +5952,7 @@
     </row>
     <row r="70">
       <c r="A70" t="str">
-        <v>SKU0158</v>
+        <v>SKU0346</v>
       </c>
       <c r="B70" t="str">
         <v>tire</v>
@@ -5985,7 +5985,7 @@
         <v>8</v>
       </c>
       <c r="L70" t="str">
-        <v>Sentury pricelist 2026</v>
+        <v>SENTURY; New SKU 2026-09-04 - เพิ่มจากไฟล์ราคา ATV Sentury (ST_July)</v>
       </c>
       <c r="M70" t="str">
         <v/>
@@ -6032,7 +6032,7 @@
     </row>
     <row r="71">
       <c r="A71" t="str">
-        <v>SKU0159</v>
+        <v>SKU0347</v>
       </c>
       <c r="B71" t="str">
         <v>tire</v>
@@ -6065,7 +6065,7 @@
         <v>8</v>
       </c>
       <c r="L71" t="str">
-        <v>Sentury pricelist 2026</v>
+        <v>SENTURY; New SKU 2026-09-04 - เพิ่มจากไฟล์ราคา ATV Sentury (ST_July)</v>
       </c>
       <c r="M71" t="str">
         <v/>
@@ -6112,7 +6112,7 @@
     </row>
     <row r="72">
       <c r="A72" t="str">
-        <v>SKU0160</v>
+        <v>SKU0348</v>
       </c>
       <c r="B72" t="str">
         <v>tire</v>
@@ -6145,7 +6145,7 @@
         <v>8</v>
       </c>
       <c r="L72" t="str">
-        <v>Sentury pricelist 2026</v>
+        <v>SENTURY; New SKU 2026-09-04 - เพิ่มจากไฟล์ราคา ATV Sentury (ST_July)</v>
       </c>
       <c r="M72" t="str">
         <v/>
@@ -6192,7 +6192,7 @@
     </row>
     <row r="73">
       <c r="A73" t="str">
-        <v>SKU0161</v>
+        <v>SKU0349</v>
       </c>
       <c r="B73" t="str">
         <v>tire</v>
@@ -6225,7 +6225,7 @@
         <v>8</v>
       </c>
       <c r="L73" t="str">
-        <v>Sentury pricelist 2026</v>
+        <v>SENTURY; New SKU 2026-09-04 - เพิ่มจากไฟล์ราคา ATV Sentury (ST_July)</v>
       </c>
       <c r="M73" t="str">
         <v/>

</xml_diff>

<commit_message>
Shorten the note field and stage the rows as a Drive spreadsheet
The per-row note repeated a long Thai sentence 72 times, which dominated
the payload; it is now "SENTURY; ATV pricelist ST_July 2026" (still
carrying WL where it applies). Brand and provenance survive in the
แบรนด์ column and the note prefix.

The same 72 rows are also uploaded to Drive as a headerless spreadsheet
next to ROKUDO Data, so the rows can be copied on a phone without opening
an attachment. Verified by exporting it back and matching the base64
against the locally generated bytes.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015Hfm3HvyUfCpK4wwTTpWTX
</commit_message>
<xml_diff>
--- a/data/rokudo_rows.xlsx
+++ b/data/rokudo_rows.xlsx
@@ -545,7 +545,7 @@
         <v>8</v>
       </c>
       <c r="L2" t="str">
-        <v>SENTURY; New SKU 2026-09-04 - เพิ่มจากไฟล์ราคา ATV Sentury (ST_July)</v>
+        <v>SENTURY; ATV pricelist ST_July 2026</v>
       </c>
       <c r="M2" t="str">
         <v/>
@@ -625,7 +625,7 @@
         <v>8</v>
       </c>
       <c r="L3" t="str">
-        <v>SENTURY; New SKU 2026-09-04 - เพิ่มจากไฟล์ราคา ATV Sentury (ST_July)</v>
+        <v>SENTURY; ATV pricelist ST_July 2026</v>
       </c>
       <c r="M3" t="str">
         <v/>
@@ -705,7 +705,7 @@
         <v>8</v>
       </c>
       <c r="L4" t="str">
-        <v>SENTURY; New SKU 2026-09-04 - เพิ่มจากไฟล์ราคา ATV Sentury (ST_July)</v>
+        <v>SENTURY; ATV pricelist ST_July 2026</v>
       </c>
       <c r="M4" t="str">
         <v/>
@@ -785,7 +785,7 @@
         <v>8</v>
       </c>
       <c r="L5" t="str">
-        <v>SENTURY; New SKU 2026-09-04 - เพิ่มจากไฟล์ราคา ATV Sentury (ST_July)</v>
+        <v>SENTURY; ATV pricelist ST_July 2026</v>
       </c>
       <c r="M5" t="str">
         <v/>
@@ -865,7 +865,7 @@
         <v>8</v>
       </c>
       <c r="L6" t="str">
-        <v>SENTURY; New SKU 2026-09-04 - เพิ่มจากไฟล์ราคา ATV Sentury (ST_July)</v>
+        <v>SENTURY; ATV pricelist ST_July 2026</v>
       </c>
       <c r="M6" t="str">
         <v/>
@@ -945,7 +945,7 @@
         <v>8</v>
       </c>
       <c r="L7" t="str">
-        <v>SENTURY; New SKU 2026-09-04 - เพิ่มจากไฟล์ราคา ATV Sentury (ST_July)</v>
+        <v>SENTURY; ATV pricelist ST_July 2026</v>
       </c>
       <c r="M7" t="str">
         <v/>
@@ -1025,7 +1025,7 @@
         <v>8</v>
       </c>
       <c r="L8" t="str">
-        <v>SENTURY; New SKU 2026-09-04 - เพิ่มจากไฟล์ราคา ATV Sentury (ST_July)</v>
+        <v>SENTURY; ATV pricelist ST_July 2026</v>
       </c>
       <c r="M8" t="str">
         <v/>
@@ -1105,7 +1105,7 @@
         <v>8</v>
       </c>
       <c r="L9" t="str">
-        <v>SENTURY; New SKU 2026-09-04 - เพิ่มจากไฟล์ราคา ATV Sentury (ST_July)</v>
+        <v>SENTURY; ATV pricelist ST_July 2026</v>
       </c>
       <c r="M9" t="str">
         <v/>
@@ -1185,7 +1185,7 @@
         <v>8</v>
       </c>
       <c r="L10" t="str">
-        <v>SENTURY; New SKU 2026-09-04 - เพิ่มจากไฟล์ราคา ATV Sentury (ST_July)</v>
+        <v>SENTURY; ATV pricelist ST_July 2026</v>
       </c>
       <c r="M10" t="str">
         <v/>
@@ -1265,7 +1265,7 @@
         <v>8</v>
       </c>
       <c r="L11" t="str">
-        <v>SENTURY; New SKU 2026-09-04 - เพิ่มจากไฟล์ราคา ATV Sentury (ST_July)</v>
+        <v>SENTURY; ATV pricelist ST_July 2026</v>
       </c>
       <c r="M11" t="str">
         <v/>
@@ -1345,7 +1345,7 @@
         <v>8</v>
       </c>
       <c r="L12" t="str">
-        <v>SENTURY; New SKU 2026-09-04 - เพิ่มจากไฟล์ราคา ATV Sentury (ST_July)</v>
+        <v>SENTURY; ATV pricelist ST_July 2026</v>
       </c>
       <c r="M12" t="str">
         <v/>
@@ -1425,7 +1425,7 @@
         <v>8</v>
       </c>
       <c r="L13" t="str">
-        <v>SENTURY; New SKU 2026-09-04 - เพิ่มจากไฟล์ราคา ATV Sentury (ST_July)</v>
+        <v>SENTURY; ATV pricelist ST_July 2026</v>
       </c>
       <c r="M13" t="str">
         <v/>
@@ -1505,7 +1505,7 @@
         <v>8</v>
       </c>
       <c r="L14" t="str">
-        <v>SENTURY; New SKU 2026-09-04 - เพิ่มจากไฟล์ราคา ATV Sentury (ST_July)</v>
+        <v>SENTURY; ATV pricelist ST_July 2026</v>
       </c>
       <c r="M14" t="str">
         <v/>
@@ -1585,7 +1585,7 @@
         <v>8</v>
       </c>
       <c r="L15" t="str">
-        <v>SENTURY; New SKU 2026-09-04 - เพิ่มจากไฟล์ราคา ATV Sentury (ST_July)</v>
+        <v>SENTURY; ATV pricelist ST_July 2026</v>
       </c>
       <c r="M15" t="str">
         <v/>
@@ -1665,7 +1665,7 @@
         <v>8</v>
       </c>
       <c r="L16" t="str">
-        <v>SENTURY; New SKU 2026-09-04 - เพิ่มจากไฟล์ราคา ATV Sentury (ST_July)</v>
+        <v>SENTURY; ATV pricelist ST_July 2026</v>
       </c>
       <c r="M16" t="str">
         <v/>
@@ -1745,7 +1745,7 @@
         <v>8</v>
       </c>
       <c r="L17" t="str">
-        <v>SENTURY; New SKU 2026-09-04 - เพิ่มจากไฟล์ราคา ATV Sentury (ST_July)</v>
+        <v>SENTURY; ATV pricelist ST_July 2026</v>
       </c>
       <c r="M17" t="str">
         <v/>
@@ -1825,7 +1825,7 @@
         <v>8</v>
       </c>
       <c r="L18" t="str">
-        <v>SENTURY; New SKU 2026-09-04 - เพิ่มจากไฟล์ราคา ATV Sentury (ST_July)</v>
+        <v>SENTURY; ATV pricelist ST_July 2026</v>
       </c>
       <c r="M18" t="str">
         <v/>
@@ -1905,7 +1905,7 @@
         <v>8</v>
       </c>
       <c r="L19" t="str">
-        <v>SENTURY; New SKU 2026-09-04 - เพิ่มจากไฟล์ราคา ATV Sentury (ST_July)</v>
+        <v>SENTURY; ATV pricelist ST_July 2026</v>
       </c>
       <c r="M19" t="str">
         <v/>
@@ -1985,7 +1985,7 @@
         <v>8</v>
       </c>
       <c r="L20" t="str">
-        <v>SENTURY; New SKU 2026-09-04 - เพิ่มจากไฟล์ราคา ATV Sentury (ST_July)</v>
+        <v>SENTURY; ATV pricelist ST_July 2026</v>
       </c>
       <c r="M20" t="str">
         <v/>
@@ -2065,7 +2065,7 @@
         <v>8</v>
       </c>
       <c r="L21" t="str">
-        <v>SENTURY; New SKU 2026-09-04 - เพิ่มจากไฟล์ราคา ATV Sentury (ST_July)</v>
+        <v>SENTURY; ATV pricelist ST_July 2026</v>
       </c>
       <c r="M21" t="str">
         <v/>
@@ -2145,7 +2145,7 @@
         <v>8</v>
       </c>
       <c r="L22" t="str">
-        <v>SENTURY; New SKU 2026-09-04 - เพิ่มจากไฟล์ราคา ATV Sentury (ST_July)</v>
+        <v>SENTURY; ATV pricelist ST_July 2026</v>
       </c>
       <c r="M22" t="str">
         <v/>
@@ -2225,7 +2225,7 @@
         <v>8</v>
       </c>
       <c r="L23" t="str">
-        <v>SENTURY; New SKU 2026-09-04 - เพิ่มจากไฟล์ราคา ATV Sentury (ST_July)</v>
+        <v>SENTURY; ATV pricelist ST_July 2026</v>
       </c>
       <c r="M23" t="str">
         <v/>
@@ -2305,7 +2305,7 @@
         <v>8</v>
       </c>
       <c r="L24" t="str">
-        <v>SENTURY; New SKU 2026-09-04 - เพิ่มจากไฟล์ราคา ATV Sentury (ST_July)</v>
+        <v>SENTURY; ATV pricelist ST_July 2026</v>
       </c>
       <c r="M24" t="str">
         <v/>
@@ -2385,7 +2385,7 @@
         <v>8</v>
       </c>
       <c r="L25" t="str">
-        <v>SENTURY; New SKU 2026-09-04 - เพิ่มจากไฟล์ราคา ATV Sentury (ST_July)</v>
+        <v>SENTURY; ATV pricelist ST_July 2026</v>
       </c>
       <c r="M25" t="str">
         <v/>
@@ -2465,7 +2465,7 @@
         <v>8</v>
       </c>
       <c r="L26" t="str">
-        <v>SENTURY; New SKU 2026-09-04 - เพิ่มจากไฟล์ราคา ATV Sentury (ST_July)</v>
+        <v>SENTURY; ATV pricelist ST_July 2026</v>
       </c>
       <c r="M26" t="str">
         <v/>
@@ -2545,7 +2545,7 @@
         <v>8</v>
       </c>
       <c r="L27" t="str">
-        <v>SENTURY; New SKU 2026-09-04 - เพิ่มจากไฟล์ราคา ATV Sentury (ST_July)</v>
+        <v>SENTURY; ATV pricelist ST_July 2026</v>
       </c>
       <c r="M27" t="str">
         <v/>
@@ -2625,7 +2625,7 @@
         <v>8</v>
       </c>
       <c r="L28" t="str">
-        <v>SENTURY; New SKU 2026-09-04 - เพิ่มจากไฟล์ราคา ATV Sentury (ST_July)</v>
+        <v>SENTURY; ATV pricelist ST_July 2026</v>
       </c>
       <c r="M28" t="str">
         <v/>
@@ -2705,7 +2705,7 @@
         <v>8</v>
       </c>
       <c r="L29" t="str">
-        <v>SENTURY; New SKU 2026-09-04 - เพิ่มจากไฟล์ราคา ATV Sentury (ST_July)</v>
+        <v>SENTURY; ATV pricelist ST_July 2026</v>
       </c>
       <c r="M29" t="str">
         <v/>
@@ -2785,7 +2785,7 @@
         <v>8</v>
       </c>
       <c r="L30" t="str">
-        <v>SENTURY; New SKU 2026-09-04 - เพิ่มจากไฟล์ราคา ATV Sentury (ST_July)</v>
+        <v>SENTURY; ATV pricelist ST_July 2026</v>
       </c>
       <c r="M30" t="str">
         <v/>
@@ -2865,7 +2865,7 @@
         <v>8</v>
       </c>
       <c r="L31" t="str">
-        <v>SENTURY; New SKU 2026-09-04 - เพิ่มจากไฟล์ราคา ATV Sentury (ST_July)</v>
+        <v>SENTURY; ATV pricelist ST_July 2026</v>
       </c>
       <c r="M31" t="str">
         <v/>
@@ -2945,7 +2945,7 @@
         <v>8</v>
       </c>
       <c r="L32" t="str">
-        <v>WL; SENTURY; New SKU 2026-09-04 - เพิ่มจากไฟล์ราคา ATV Sentury (ST_July)</v>
+        <v>WL; SENTURY; ATV pricelist ST_July 2026</v>
       </c>
       <c r="M32" t="str">
         <v/>
@@ -3025,7 +3025,7 @@
         <v>8</v>
       </c>
       <c r="L33" t="str">
-        <v>WL; SENTURY; New SKU 2026-09-04 - เพิ่มจากไฟล์ราคา ATV Sentury (ST_July)</v>
+        <v>WL; SENTURY; ATV pricelist ST_July 2026</v>
       </c>
       <c r="M33" t="str">
         <v/>
@@ -3105,7 +3105,7 @@
         <v>8</v>
       </c>
       <c r="L34" t="str">
-        <v>WL; SENTURY; New SKU 2026-09-04 - เพิ่มจากไฟล์ราคา ATV Sentury (ST_July)</v>
+        <v>WL; SENTURY; ATV pricelist ST_July 2026</v>
       </c>
       <c r="M34" t="str">
         <v/>
@@ -3185,7 +3185,7 @@
         <v>8</v>
       </c>
       <c r="L35" t="str">
-        <v>WL; SENTURY; New SKU 2026-09-04 - เพิ่มจากไฟล์ราคา ATV Sentury (ST_July)</v>
+        <v>WL; SENTURY; ATV pricelist ST_July 2026</v>
       </c>
       <c r="M35" t="str">
         <v/>
@@ -3265,7 +3265,7 @@
         <v>8</v>
       </c>
       <c r="L36" t="str">
-        <v>WL; SENTURY; New SKU 2026-09-04 - เพิ่มจากไฟล์ราคา ATV Sentury (ST_July)</v>
+        <v>WL; SENTURY; ATV pricelist ST_July 2026</v>
       </c>
       <c r="M36" t="str">
         <v/>
@@ -3345,7 +3345,7 @@
         <v>8</v>
       </c>
       <c r="L37" t="str">
-        <v>WL; SENTURY; New SKU 2026-09-04 - เพิ่มจากไฟล์ราคา ATV Sentury (ST_July)</v>
+        <v>WL; SENTURY; ATV pricelist ST_July 2026</v>
       </c>
       <c r="M37" t="str">
         <v/>
@@ -3425,7 +3425,7 @@
         <v>8</v>
       </c>
       <c r="L38" t="str">
-        <v>WL; SENTURY; New SKU 2026-09-04 - เพิ่มจากไฟล์ราคา ATV Sentury (ST_July)</v>
+        <v>WL; SENTURY; ATV pricelist ST_July 2026</v>
       </c>
       <c r="M38" t="str">
         <v/>
@@ -3505,7 +3505,7 @@
         <v>8</v>
       </c>
       <c r="L39" t="str">
-        <v>WL; SENTURY; New SKU 2026-09-04 - เพิ่มจากไฟล์ราคา ATV Sentury (ST_July)</v>
+        <v>WL; SENTURY; ATV pricelist ST_July 2026</v>
       </c>
       <c r="M39" t="str">
         <v/>
@@ -3585,7 +3585,7 @@
         <v>8</v>
       </c>
       <c r="L40" t="str">
-        <v>WL; SENTURY; New SKU 2026-09-04 - เพิ่มจากไฟล์ราคา ATV Sentury (ST_July)</v>
+        <v>WL; SENTURY; ATV pricelist ST_July 2026</v>
       </c>
       <c r="M40" t="str">
         <v/>
@@ -3665,7 +3665,7 @@
         <v>8</v>
       </c>
       <c r="L41" t="str">
-        <v>WL; SENTURY; New SKU 2026-09-04 - เพิ่มจากไฟล์ราคา ATV Sentury (ST_July)</v>
+        <v>WL; SENTURY; ATV pricelist ST_July 2026</v>
       </c>
       <c r="M41" t="str">
         <v/>
@@ -3745,7 +3745,7 @@
         <v>8</v>
       </c>
       <c r="L42" t="str">
-        <v>WL; SENTURY; New SKU 2026-09-04 - เพิ่มจากไฟล์ราคา ATV Sentury (ST_July)</v>
+        <v>WL; SENTURY; ATV pricelist ST_July 2026</v>
       </c>
       <c r="M42" t="str">
         <v/>
@@ -3825,7 +3825,7 @@
         <v>8</v>
       </c>
       <c r="L43" t="str">
-        <v>WL; SENTURY; New SKU 2026-09-04 - เพิ่มจากไฟล์ราคา ATV Sentury (ST_July)</v>
+        <v>WL; SENTURY; ATV pricelist ST_July 2026</v>
       </c>
       <c r="M43" t="str">
         <v/>
@@ -3905,7 +3905,7 @@
         <v>8</v>
       </c>
       <c r="L44" t="str">
-        <v>WL; SENTURY; New SKU 2026-09-04 - เพิ่มจากไฟล์ราคา ATV Sentury (ST_July)</v>
+        <v>WL; SENTURY; ATV pricelist ST_July 2026</v>
       </c>
       <c r="M44" t="str">
         <v/>
@@ -3985,7 +3985,7 @@
         <v>8</v>
       </c>
       <c r="L45" t="str">
-        <v>SENTURY; New SKU 2026-09-04 - เพิ่มจากไฟล์ราคา ATV Sentury (ST_July)</v>
+        <v>SENTURY; ATV pricelist ST_July 2026</v>
       </c>
       <c r="M45" t="str">
         <v/>
@@ -4065,7 +4065,7 @@
         <v>8</v>
       </c>
       <c r="L46" t="str">
-        <v>SENTURY; New SKU 2026-09-04 - เพิ่มจากไฟล์ราคา ATV Sentury (ST_July)</v>
+        <v>SENTURY; ATV pricelist ST_July 2026</v>
       </c>
       <c r="M46" t="str">
         <v/>
@@ -4145,7 +4145,7 @@
         <v>8</v>
       </c>
       <c r="L47" t="str">
-        <v>SENTURY; New SKU 2026-09-04 - เพิ่มจากไฟล์ราคา ATV Sentury (ST_July)</v>
+        <v>SENTURY; ATV pricelist ST_July 2026</v>
       </c>
       <c r="M47" t="str">
         <v/>
@@ -4225,7 +4225,7 @@
         <v>8</v>
       </c>
       <c r="L48" t="str">
-        <v>SENTURY; New SKU 2026-09-04 - เพิ่มจากไฟล์ราคา ATV Sentury (ST_July)</v>
+        <v>SENTURY; ATV pricelist ST_July 2026</v>
       </c>
       <c r="M48" t="str">
         <v/>
@@ -4305,7 +4305,7 @@
         <v>8</v>
       </c>
       <c r="L49" t="str">
-        <v>SENTURY; New SKU 2026-09-04 - เพิ่มจากไฟล์ราคา ATV Sentury (ST_July)</v>
+        <v>SENTURY; ATV pricelist ST_July 2026</v>
       </c>
       <c r="M49" t="str">
         <v/>
@@ -4385,7 +4385,7 @@
         <v>8</v>
       </c>
       <c r="L50" t="str">
-        <v>SENTURY; New SKU 2026-09-04 - เพิ่มจากไฟล์ราคา ATV Sentury (ST_July)</v>
+        <v>SENTURY; ATV pricelist ST_July 2026</v>
       </c>
       <c r="M50" t="str">
         <v/>
@@ -4465,7 +4465,7 @@
         <v>8</v>
       </c>
       <c r="L51" t="str">
-        <v>SENTURY; New SKU 2026-09-04 - เพิ่มจากไฟล์ราคา ATV Sentury (ST_July)</v>
+        <v>SENTURY; ATV pricelist ST_July 2026</v>
       </c>
       <c r="M51" t="str">
         <v/>
@@ -4545,7 +4545,7 @@
         <v>8</v>
       </c>
       <c r="L52" t="str">
-        <v>SENTURY; New SKU 2026-09-04 - เพิ่มจากไฟล์ราคา ATV Sentury (ST_July)</v>
+        <v>SENTURY; ATV pricelist ST_July 2026</v>
       </c>
       <c r="M52" t="str">
         <v/>
@@ -4625,7 +4625,7 @@
         <v>8</v>
       </c>
       <c r="L53" t="str">
-        <v>SENTURY; New SKU 2026-09-04 - เพิ่มจากไฟล์ราคา ATV Sentury (ST_July)</v>
+        <v>SENTURY; ATV pricelist ST_July 2026</v>
       </c>
       <c r="M53" t="str">
         <v/>
@@ -4705,7 +4705,7 @@
         <v>8</v>
       </c>
       <c r="L54" t="str">
-        <v>SENTURY; New SKU 2026-09-04 - เพิ่มจากไฟล์ราคา ATV Sentury (ST_July)</v>
+        <v>SENTURY; ATV pricelist ST_July 2026</v>
       </c>
       <c r="M54" t="str">
         <v/>
@@ -4785,7 +4785,7 @@
         <v>8</v>
       </c>
       <c r="L55" t="str">
-        <v>SENTURY; New SKU 2026-09-04 - เพิ่มจากไฟล์ราคา ATV Sentury (ST_July)</v>
+        <v>SENTURY; ATV pricelist ST_July 2026</v>
       </c>
       <c r="M55" t="str">
         <v/>
@@ -4865,7 +4865,7 @@
         <v>8</v>
       </c>
       <c r="L56" t="str">
-        <v>SENTURY; New SKU 2026-09-04 - เพิ่มจากไฟล์ราคา ATV Sentury (ST_July)</v>
+        <v>SENTURY; ATV pricelist ST_July 2026</v>
       </c>
       <c r="M56" t="str">
         <v/>
@@ -4945,7 +4945,7 @@
         <v>8</v>
       </c>
       <c r="L57" t="str">
-        <v>SENTURY; New SKU 2026-09-04 - เพิ่มจากไฟล์ราคา ATV Sentury (ST_July)</v>
+        <v>SENTURY; ATV pricelist ST_July 2026</v>
       </c>
       <c r="M57" t="str">
         <v/>
@@ -5025,7 +5025,7 @@
         <v>8</v>
       </c>
       <c r="L58" t="str">
-        <v>SENTURY; New SKU 2026-09-04 - เพิ่มจากไฟล์ราคา ATV Sentury (ST_July)</v>
+        <v>SENTURY; ATV pricelist ST_July 2026</v>
       </c>
       <c r="M58" t="str">
         <v/>
@@ -5105,7 +5105,7 @@
         <v>8</v>
       </c>
       <c r="L59" t="str">
-        <v>SENTURY; New SKU 2026-09-04 - เพิ่มจากไฟล์ราคา ATV Sentury (ST_July)</v>
+        <v>SENTURY; ATV pricelist ST_July 2026</v>
       </c>
       <c r="M59" t="str">
         <v/>
@@ -5185,7 +5185,7 @@
         <v>8</v>
       </c>
       <c r="L60" t="str">
-        <v>SENTURY; New SKU 2026-09-04 - เพิ่มจากไฟล์ราคา ATV Sentury (ST_July)</v>
+        <v>SENTURY; ATV pricelist ST_July 2026</v>
       </c>
       <c r="M60" t="str">
         <v/>
@@ -5265,7 +5265,7 @@
         <v>8</v>
       </c>
       <c r="L61" t="str">
-        <v>SENTURY; New SKU 2026-09-04 - เพิ่มจากไฟล์ราคา ATV Sentury (ST_July)</v>
+        <v>SENTURY; ATV pricelist ST_July 2026</v>
       </c>
       <c r="M61" t="str">
         <v/>
@@ -5345,7 +5345,7 @@
         <v>8</v>
       </c>
       <c r="L62" t="str">
-        <v>SENTURY; New SKU 2026-09-04 - เพิ่มจากไฟล์ราคา ATV Sentury (ST_July)</v>
+        <v>SENTURY; ATV pricelist ST_July 2026</v>
       </c>
       <c r="M62" t="str">
         <v/>
@@ -5425,7 +5425,7 @@
         <v>8</v>
       </c>
       <c r="L63" t="str">
-        <v>SENTURY; New SKU 2026-09-04 - เพิ่มจากไฟล์ราคา ATV Sentury (ST_July)</v>
+        <v>SENTURY; ATV pricelist ST_July 2026</v>
       </c>
       <c r="M63" t="str">
         <v/>
@@ -5505,7 +5505,7 @@
         <v>8</v>
       </c>
       <c r="L64" t="str">
-        <v>SENTURY; New SKU 2026-09-04 - เพิ่มจากไฟล์ราคา ATV Sentury (ST_July)</v>
+        <v>SENTURY; ATV pricelist ST_July 2026</v>
       </c>
       <c r="M64" t="str">
         <v/>
@@ -5585,7 +5585,7 @@
         <v>8</v>
       </c>
       <c r="L65" t="str">
-        <v>SENTURY; New SKU 2026-09-04 - เพิ่มจากไฟล์ราคา ATV Sentury (ST_July)</v>
+        <v>SENTURY; ATV pricelist ST_July 2026</v>
       </c>
       <c r="M65" t="str">
         <v/>
@@ -5665,7 +5665,7 @@
         <v>8</v>
       </c>
       <c r="L66" t="str">
-        <v>SENTURY; New SKU 2026-09-04 - เพิ่มจากไฟล์ราคา ATV Sentury (ST_July)</v>
+        <v>SENTURY; ATV pricelist ST_July 2026</v>
       </c>
       <c r="M66" t="str">
         <v/>
@@ -5745,7 +5745,7 @@
         <v>8</v>
       </c>
       <c r="L67" t="str">
-        <v>SENTURY; New SKU 2026-09-04 - เพิ่มจากไฟล์ราคา ATV Sentury (ST_July)</v>
+        <v>SENTURY; ATV pricelist ST_July 2026</v>
       </c>
       <c r="M67" t="str">
         <v/>
@@ -5825,7 +5825,7 @@
         <v>8</v>
       </c>
       <c r="L68" t="str">
-        <v>SENTURY; New SKU 2026-09-04 - เพิ่มจากไฟล์ราคา ATV Sentury (ST_July)</v>
+        <v>SENTURY; ATV pricelist ST_July 2026</v>
       </c>
       <c r="M68" t="str">
         <v/>
@@ -5905,7 +5905,7 @@
         <v>8</v>
       </c>
       <c r="L69" t="str">
-        <v>SENTURY; New SKU 2026-09-04 - เพิ่มจากไฟล์ราคา ATV Sentury (ST_July)</v>
+        <v>SENTURY; ATV pricelist ST_July 2026</v>
       </c>
       <c r="M69" t="str">
         <v/>
@@ -5985,7 +5985,7 @@
         <v>8</v>
       </c>
       <c r="L70" t="str">
-        <v>SENTURY; New SKU 2026-09-04 - เพิ่มจากไฟล์ราคา ATV Sentury (ST_July)</v>
+        <v>SENTURY; ATV pricelist ST_July 2026</v>
       </c>
       <c r="M70" t="str">
         <v/>
@@ -6065,7 +6065,7 @@
         <v>8</v>
       </c>
       <c r="L71" t="str">
-        <v>SENTURY; New SKU 2026-09-04 - เพิ่มจากไฟล์ราคา ATV Sentury (ST_July)</v>
+        <v>SENTURY; ATV pricelist ST_July 2026</v>
       </c>
       <c r="M71" t="str">
         <v/>
@@ -6145,7 +6145,7 @@
         <v>8</v>
       </c>
       <c r="L72" t="str">
-        <v>SENTURY; New SKU 2026-09-04 - เพิ่มจากไฟล์ราคา ATV Sentury (ST_July)</v>
+        <v>SENTURY; ATV pricelist ST_July 2026</v>
       </c>
       <c r="M72" t="str">
         <v/>
@@ -6225,7 +6225,7 @@
         <v>8</v>
       </c>
       <c r="L73" t="str">
-        <v>SENTURY; New SKU 2026-09-04 - เพิ่มจากไฟล์ราคา ATV Sentury (ST_July)</v>
+        <v>SENTURY; ATV pricelist ST_July 2026</v>
       </c>
       <c r="M73" t="str">
         <v/>

</xml_diff>